<commit_message>
Minor foramting issu to data dictonry fixed
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F76268E0-3C5D-9F4D-81FD-85C0F9E5DF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA09C7AA-3967-FE4A-9DE6-CF36BDD7C097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
@@ -737,9 +737,6 @@
     <t>trt_description</t>
   </si>
   <si>
-    <t>as in: control: format: character</t>
-  </si>
-  <si>
     <t>as in: benjamin.hlina@gmail.com - valid email address; format: character</t>
   </si>
   <si>
@@ -1061,10 +1058,13 @@
     <t>as in: -150.40 ‰; numeric: integer; places to 2 decimals</t>
   </si>
   <si>
-    <t>as in: -14.50 ‰; format:numeric; places to 2 decimals</t>
+    <t xml:space="preserve">as in: 3.80; format: numeric; place to 2 decimals </t>
   </si>
   <si>
-    <t xml:space="preserve">as in: 3.80; format: numeric; place to 2 decimals </t>
+    <t>as in: control; format: character</t>
+  </si>
+  <si>
+    <t>as in: -14.50 ‰; format: numeric; places to 2 decimals</t>
   </si>
 </sst>
 </file>
@@ -1751,7 +1751,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
@@ -1759,7 +1759,7 @@
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="45" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -1779,63 +1779,63 @@
         <v>2</v>
       </c>
       <c r="E4" s="44" t="s">
+        <v>204</v>
+      </c>
+      <c r="F4" s="44" t="s">
         <v>205</v>
       </c>
-      <c r="F4" s="44" t="s">
-        <v>206</v>
-      </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>184</v>
-      </c>
       <c r="D5" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="E5" s="31"/>
       <c r="F5" s="31"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E6" s="31"/>
       <c r="F6" s="31"/>
     </row>
     <row r="7" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C7" s="19" t="s">
         <v>149</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E7" s="31"/>
       <c r="F7" s="31"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>4</v>
@@ -1851,7 +1851,7 @@
     </row>
     <row r="9" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>66</v>
@@ -1863,13 +1863,13 @@
         <v>78</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>67</v>
@@ -1885,7 +1885,7 @@
     </row>
     <row r="11" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A11" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>68</v>
@@ -1901,25 +1901,25 @@
     </row>
     <row r="12" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B12" s="28" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D12" s="25" t="s">
         <v>81</v>
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="34" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>70</v>
@@ -1932,12 +1932,12 @@
       </c>
       <c r="E13" s="31"/>
       <c r="F13" s="34" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B14" s="28" t="s">
         <v>115</v>
@@ -1953,7 +1953,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B15" s="25" t="s">
         <v>71</v>
@@ -1969,7 +1969,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B16" s="25" t="s">
         <v>116</v>
@@ -1985,7 +1985,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B17" s="25" t="s">
         <v>117</v>
@@ -2001,7 +2001,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>72</v>
@@ -2017,7 +2017,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>73</v>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="20" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>74</v>
@@ -2049,7 +2049,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B21" s="25" t="s">
         <v>145</v>
@@ -2065,7 +2065,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="26" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B22" s="25" t="s">
         <v>75</v>
@@ -2183,14 +2183,14 @@
         <v>6</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D29" s="31" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="34" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -2198,7 +2198,7 @@
         <v>124</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C30" s="31" t="s">
         <v>140</v>
@@ -2249,13 +2249,13 @@
         <v>7</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D33" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E33" s="31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F33" s="31"/>
     </row>
@@ -2267,13 +2267,13 @@
         <v>8</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D34" s="31" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E34" s="34" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F34" s="31"/>
     </row>
@@ -2291,7 +2291,7 @@
         <v>114</v>
       </c>
       <c r="E35" s="31" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F35" s="31"/>
     </row>
@@ -2303,10 +2303,10 @@
         <v>162</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>163</v>
+        <v>257</v>
       </c>
       <c r="D36" s="34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
@@ -2316,10 +2316,10 @@
         <v>124</v>
       </c>
       <c r="B37" s="31" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D37" s="31" t="s">
         <v>40</v>
@@ -2335,10 +2335,10 @@
         <v>99</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D38" s="31" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E38" s="31"/>
       <c r="F38" s="31"/>
@@ -2351,13 +2351,13 @@
         <v>100</v>
       </c>
       <c r="C39" s="31" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D39" s="34" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E39" s="31" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F39" s="31"/>
     </row>
@@ -2366,13 +2366,13 @@
         <v>124</v>
       </c>
       <c r="B40" s="31" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C40" s="31" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D40" s="31" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="E40" s="31"/>
       <c r="F40" s="31"/>
@@ -2382,16 +2382,16 @@
         <v>124</v>
       </c>
       <c r="B41" s="33" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C41" s="31" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D41" s="34" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="E41" s="34" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="F41" s="31"/>
     </row>
@@ -2400,7 +2400,7 @@
         <v>124</v>
       </c>
       <c r="B42" s="31" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C42" s="31" t="s">
         <v>59</v>
@@ -2425,7 +2425,7 @@
         <v>12</v>
       </c>
       <c r="E43" s="34" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F43" s="31"/>
     </row>
@@ -2443,7 +2443,7 @@
         <v>64</v>
       </c>
       <c r="E44" s="31" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F44" s="31"/>
     </row>
@@ -2490,7 +2490,7 @@
         <v>159</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E47" s="31"/>
       <c r="F47" s="31"/>
@@ -2506,7 +2506,7 @@
         <v>52</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E48" s="31"/>
       <c r="F48" s="31"/>
@@ -2522,7 +2522,7 @@
         <v>143</v>
       </c>
       <c r="D49" s="31" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="E49" s="31"/>
       <c r="F49" s="31"/>
@@ -2538,11 +2538,11 @@
         <v>156</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E50" s="31"/>
       <c r="F50" s="34" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="56" x14ac:dyDescent="0.2">
@@ -2556,11 +2556,11 @@
         <v>157</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E51" s="31"/>
       <c r="F51" s="34" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="84" x14ac:dyDescent="0.2">
@@ -2571,13 +2571,13 @@
         <v>55</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E52" s="34" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F52" s="31"/>
     </row>
@@ -2608,7 +2608,7 @@
         <v>146</v>
       </c>
       <c r="D54" s="31" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E54" s="31"/>
       <c r="F54" s="31"/>
@@ -2627,7 +2627,7 @@
         <v>104</v>
       </c>
       <c r="E55" s="31" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="F55" s="31"/>
     </row>
@@ -2639,10 +2639,10 @@
         <v>125</v>
       </c>
       <c r="C56" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D56" s="31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="E56" s="31"/>
       <c r="F56" s="31"/>
@@ -2661,7 +2661,7 @@
         <v>105</v>
       </c>
       <c r="E57" s="31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="F57" s="31"/>
     </row>
@@ -2689,10 +2689,10 @@
         <v>123</v>
       </c>
       <c r="C59" s="31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D59" s="31" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E59" s="31"/>
       <c r="F59" s="31"/>
@@ -2705,7 +2705,7 @@
         <v>126</v>
       </c>
       <c r="C60" s="31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D60" s="34" t="s">
         <v>129</v>
@@ -2721,7 +2721,7 @@
         <v>127</v>
       </c>
       <c r="C61" s="31" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D61" s="34" t="s">
         <v>130</v>
@@ -2737,7 +2737,7 @@
         <v>28</v>
       </c>
       <c r="C62" s="31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D62" s="31" t="s">
         <v>41</v>
@@ -2753,7 +2753,7 @@
         <v>30</v>
       </c>
       <c r="C63" s="31" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D63" s="31" t="s">
         <v>42</v>
@@ -2769,7 +2769,7 @@
         <v>31</v>
       </c>
       <c r="C64" s="31" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D64" s="31" t="s">
         <v>43</v>
@@ -2785,7 +2785,7 @@
         <v>32</v>
       </c>
       <c r="C65" s="31" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D65" s="31" t="s">
         <v>44</v>
@@ -2801,7 +2801,7 @@
         <v>33</v>
       </c>
       <c r="C66" s="31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D66" s="31" t="s">
         <v>45</v>
@@ -2817,7 +2817,7 @@
         <v>34</v>
       </c>
       <c r="C67" s="31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D67" s="31" t="s">
         <v>46</v>
@@ -2830,16 +2830,16 @@
         <v>38</v>
       </c>
       <c r="B68" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="C68" s="31" t="s">
         <v>187</v>
       </c>
-      <c r="C68" s="31" t="s">
-        <v>188</v>
-      </c>
       <c r="D68" s="34" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="E68" s="31" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="F68" s="31"/>
     </row>
@@ -2851,7 +2851,7 @@
         <v>35</v>
       </c>
       <c r="C69" s="31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D69" s="31" t="s">
         <v>49</v>
@@ -2867,7 +2867,7 @@
         <v>36</v>
       </c>
       <c r="C70" s="31" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D70" s="31" t="s">
         <v>50</v>
@@ -2883,7 +2883,7 @@
         <v>37</v>
       </c>
       <c r="C71" s="31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D71" s="31" t="s">
         <v>51</v>
@@ -2896,13 +2896,13 @@
         <v>38</v>
       </c>
       <c r="B72" s="31" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C72" s="31" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D72" s="31" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E72" s="31"/>
       <c r="F72" s="31"/>
@@ -2912,13 +2912,13 @@
         <v>38</v>
       </c>
       <c r="B73" s="31" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C73" s="31" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D73" s="31" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="E73" s="31"/>
       <c r="F73" s="31"/>
@@ -2931,7 +2931,7 @@
         <v>131</v>
       </c>
       <c r="C74" s="31" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D74" s="31" t="s">
         <v>132</v>
@@ -2960,12 +2960,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -2981,18 +2981,18 @@
       <c r="B3" s="46"/>
       <c r="C3" s="46"/>
       <c r="D3" s="11" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="13" t="s">
         <v>180</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -3026,12 +3026,12 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="10" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -3052,7 +3052,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>66</v>
@@ -44038,12 +44038,12 @@
   <sheetData>
     <row r="1" spans="1:53" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
@@ -44087,10 +44087,10 @@
         <v>65</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>53</v>
@@ -44102,10 +44102,10 @@
         <v>118</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="I5" s="39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="J5" s="37" t="s">
         <v>15</v>
@@ -44114,7 +44114,7 @@
         <v>107</v>
       </c>
       <c r="L5" s="37" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="M5" s="37" t="s">
         <v>8</v>
@@ -44126,7 +44126,7 @@
         <v>162</v>
       </c>
       <c r="P5" s="37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="Q5" s="37" t="s">
         <v>99</v>
@@ -44135,13 +44135,13 @@
         <v>100</v>
       </c>
       <c r="S5" s="37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T5" s="40" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="U5" s="40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="V5" s="39" t="s">
         <v>9</v>
@@ -44165,10 +44165,10 @@
         <v>21</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AE5" s="42" t="s">
         <v>55</v>
@@ -44219,7 +44219,7 @@
         <v>34</v>
       </c>
       <c r="AU5" s="37" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="AV5" s="37" t="s">
         <v>35</v>
@@ -44231,10 +44231,10 @@
         <v>37</v>
       </c>
       <c r="AY5" s="37" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AZ5" s="37" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="BA5" s="37" t="s">
         <v>131</v>

</xml_diff>

<commit_message>
removed addtional columns in dd
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA09C7AA-3967-FE4A-9DE6-CF36BDD7C097}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94E3D2A-47E0-E844-8BF2-DA05771D155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="tbl_samples" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_dictionary!$A$4:$D$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">data_dictionary!$A$4:$D$73</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="257">
   <si>
     <t>Field Name</t>
   </si>
@@ -581,9 +581,6 @@
     <t>Genus of the organism</t>
   </si>
   <si>
-    <t xml:space="preserve">Family of the organism </t>
-  </si>
-  <si>
     <t>Date that the sample was collected</t>
   </si>
   <si>
@@ -672,9 +669,6 @@
   </si>
   <si>
     <t>as in: Salvelinus; format: character</t>
-  </si>
-  <si>
-    <t>as in: Salmonidae; format: character</t>
   </si>
   <si>
     <t>as in 30 m; format: integer</t>
@@ -1737,7 +1731,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCDB0B4B-8041-E244-B061-95D35DE0CD3B}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="1" customWidth="1"/>
@@ -1751,7 +1745,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="45" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B1" s="45"/>
       <c r="C1" s="45"/>
@@ -1759,7 +1753,7 @@
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="45" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -1779,63 +1773,63 @@
         <v>2</v>
       </c>
       <c r="E4" s="44" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="F4" s="44" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="23" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E5" s="31"/>
       <c r="F5" s="31"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="23" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C6" s="19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D6" s="25" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="E6" s="31"/>
       <c r="F6" s="31"/>
     </row>
     <row r="7" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A7" s="23" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D7" s="25" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="E7" s="31"/>
       <c r="F7" s="31"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="26" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B8" s="27" t="s">
         <v>4</v>
@@ -1851,31 +1845,31 @@
     </row>
     <row r="9" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A9" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B9" s="28" t="s">
         <v>66</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>78</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A10" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B10" s="28" t="s">
         <v>67</v>
       </c>
       <c r="C10" s="19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D10" s="25" t="s">
         <v>79</v>
@@ -1885,13 +1879,13 @@
     </row>
     <row r="11" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A11" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B11" s="25" t="s">
         <v>68</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D11" s="25" t="s">
         <v>80</v>
@@ -1901,46 +1895,46 @@
     </row>
     <row r="12" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A12" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B12" s="28" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D12" s="25" t="s">
         <v>81</v>
       </c>
       <c r="E12" s="31"/>
       <c r="F12" s="34" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A13" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B13" s="25" t="s">
         <v>70</v>
       </c>
       <c r="C13" s="19" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D13" s="25" t="s">
         <v>82</v>
       </c>
       <c r="E13" s="31"/>
       <c r="F13" s="34" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C14" s="25" t="s">
         <v>83</v>
@@ -1953,13 +1947,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B15" s="25" t="s">
         <v>71</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D15" s="25" t="s">
         <v>85</v>
@@ -1969,39 +1963,39 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B16" s="25" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C16" s="25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D16" s="25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E16" s="31"/>
       <c r="F16" s="31"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B17" s="25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E17" s="31"/>
       <c r="F17" s="31"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B18" s="25" t="s">
         <v>72</v>
@@ -2017,7 +2011,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B19" s="25" t="s">
         <v>73</v>
@@ -2033,7 +2027,7 @@
     </row>
     <row r="20" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A20" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B20" s="25" t="s">
         <v>74</v>
@@ -2049,10 +2043,10 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="C21" s="19" t="s">
         <v>92</v>
@@ -2065,13 +2059,13 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="26" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B22" s="25" t="s">
         <v>75</v>
       </c>
       <c r="C22" s="25" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D22" s="25" t="s">
         <v>94</v>
@@ -2081,7 +2075,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="29" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>14</v>
@@ -2097,10 +2091,10 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" s="31" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C24" s="31" t="s">
         <v>39</v>
@@ -2113,45 +2107,45 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B25" s="32" t="s">
         <v>57</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E25" s="31"/>
       <c r="F25" s="31"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B26" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="31" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D26" s="31" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E26" s="31"/>
       <c r="F26" s="31"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B27" s="31" t="s">
         <v>97</v>
       </c>
       <c r="C27" s="31" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="D27" s="31" t="s">
         <v>98</v>
@@ -2161,63 +2155,63 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B28" s="31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C28" s="31" t="s">
         <v>83</v>
       </c>
       <c r="D28" s="31" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E28" s="31"/>
       <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" ht="42" x14ac:dyDescent="0.2">
       <c r="A29" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B29" s="33" t="s">
         <v>6</v>
       </c>
       <c r="C29" s="31" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D29" s="31" t="s">
         <v>11</v>
       </c>
       <c r="E29" s="31"/>
       <c r="F29" s="34" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B30" s="33" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C30" s="31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D30" s="31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E30" s="31"/>
       <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B31" s="31" t="s">
         <v>15</v>
       </c>
       <c r="C31" s="31" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D31" s="31" t="s">
         <v>110</v>
@@ -2227,238 +2221,238 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B32" s="31" t="s">
-        <v>107</v>
+        <v>7</v>
       </c>
       <c r="C32" s="31" t="s">
-        <v>142</v>
+        <v>201</v>
       </c>
       <c r="D32" s="31" t="s">
-        <v>111</v>
+        <v>206</v>
       </c>
-      <c r="E32" s="31"/>
+      <c r="E32" s="31" t="s">
+        <v>204</v>
+      </c>
       <c r="F32" s="31"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A33" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B33" s="31" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C33" s="31" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D33" s="31" t="s">
-        <v>208</v>
+        <v>182</v>
       </c>
-      <c r="E33" s="31" t="s">
-        <v>206</v>
+      <c r="E33" s="34" t="s">
+        <v>207</v>
       </c>
       <c r="F33" s="31"/>
     </row>
-    <row r="34" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
-      <c r="B34" s="31" t="s">
-        <v>8</v>
+      <c r="B34" s="33" t="s">
+        <v>13</v>
       </c>
       <c r="C34" s="31" t="s">
-        <v>207</v>
+        <v>47</v>
       </c>
-      <c r="D34" s="31" t="s">
-        <v>184</v>
+      <c r="D34" s="34" t="s">
+        <v>113</v>
       </c>
-      <c r="E34" s="34" t="s">
-        <v>209</v>
+      <c r="E34" s="31" t="s">
+        <v>213</v>
       </c>
       <c r="F34" s="31"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A35" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
-      <c r="B35" s="33" t="s">
-        <v>13</v>
+      <c r="B35" s="31" t="s">
+        <v>160</v>
       </c>
       <c r="C35" s="31" t="s">
-        <v>47</v>
+        <v>255</v>
       </c>
       <c r="D35" s="34" t="s">
-        <v>114</v>
+        <v>214</v>
       </c>
-      <c r="E35" s="31" t="s">
-        <v>215</v>
-      </c>
+      <c r="E35" s="31"/>
       <c r="F35" s="31"/>
     </row>
-    <row r="36" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B36" s="31" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="C36" s="31" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
-      <c r="D36" s="34" t="s">
-        <v>216</v>
+      <c r="D36" s="31" t="s">
+        <v>40</v>
       </c>
       <c r="E36" s="31"/>
       <c r="F36" s="31"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="31" t="s">
-        <v>124</v>
+        <v>159</v>
       </c>
       <c r="B37" s="31" t="s">
-        <v>175</v>
+        <v>99</v>
       </c>
       <c r="C37" s="31" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D37" s="31" t="s">
-        <v>40</v>
+        <v>183</v>
       </c>
       <c r="E37" s="31"/>
       <c r="F37" s="31"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A38" s="31" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B38" s="31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C38" s="31" t="s">
-        <v>244</v>
+        <v>217</v>
       </c>
-      <c r="D38" s="31" t="s">
-        <v>185</v>
+      <c r="D38" s="34" t="s">
+        <v>216</v>
       </c>
-      <c r="E38" s="31"/>
+      <c r="E38" s="31" t="s">
+        <v>218</v>
+      </c>
       <c r="F38" s="31"/>
     </row>
-    <row r="39" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="31" t="s">
-        <v>161</v>
+        <v>123</v>
       </c>
       <c r="B39" s="31" t="s">
-        <v>100</v>
+        <v>174</v>
       </c>
       <c r="C39" s="31" t="s">
+        <v>243</v>
+      </c>
+      <c r="D39" s="31" t="s">
+        <v>215</v>
+      </c>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
+    </row>
+    <row r="40" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+      <c r="A40" s="31" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" s="33" t="s">
+        <v>192</v>
+      </c>
+      <c r="C40" s="31" t="s">
+        <v>194</v>
+      </c>
+      <c r="D40" s="34" t="s">
         <v>219</v>
       </c>
-      <c r="D39" s="34" t="s">
-        <v>218</v>
+      <c r="E40" s="34" t="s">
+        <v>240</v>
       </c>
-      <c r="E39" s="31" t="s">
-        <v>220</v>
+      <c r="F40" s="31"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="31" t="s">
+        <v>123</v>
       </c>
-      <c r="F39" s="31"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A40" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="B40" s="31" t="s">
-        <v>176</v>
-      </c>
-      <c r="C40" s="31" t="s">
-        <v>245</v>
-      </c>
-      <c r="D40" s="31" t="s">
-        <v>217</v>
-      </c>
-      <c r="E40" s="31"/>
-      <c r="F40" s="31"/>
-    </row>
-    <row r="41" spans="1:6" ht="28" x14ac:dyDescent="0.2">
-      <c r="A41" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="B41" s="33" t="s">
-        <v>194</v>
+      <c r="B41" s="31" t="s">
+        <v>193</v>
       </c>
       <c r="C41" s="31" t="s">
-        <v>196</v>
+        <v>59</v>
       </c>
-      <c r="D41" s="34" t="s">
-        <v>221</v>
+      <c r="D41" s="31" t="s">
+        <v>60</v>
       </c>
-      <c r="E41" s="34" t="s">
-        <v>242</v>
+      <c r="E41" s="31"/>
+      <c r="F41" s="31"/>
+    </row>
+    <row r="42" spans="1:6" ht="84" x14ac:dyDescent="0.2">
+      <c r="A42" s="31" t="s">
+        <v>123</v>
       </c>
-      <c r="F41" s="31"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="31" t="s">
-        <v>124</v>
-      </c>
-      <c r="B42" s="31" t="s">
-        <v>195</v>
+      <c r="B42" s="33" t="s">
+        <v>9</v>
       </c>
       <c r="C42" s="31" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D42" s="31" t="s">
-        <v>60</v>
+        <v>12</v>
       </c>
-      <c r="E42" s="31"/>
+      <c r="E42" s="34" t="s">
+        <v>232</v>
+      </c>
       <c r="F42" s="31"/>
     </row>
-    <row r="43" spans="1:6" ht="84" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="31" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B43" s="33" t="s">
-        <v>9</v>
+        <v>62</v>
       </c>
       <c r="C43" s="31" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D43" s="31" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
-      <c r="E43" s="34" t="s">
-        <v>234</v>
+      <c r="E43" s="31" t="s">
+        <v>231</v>
       </c>
       <c r="F43" s="31"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>124</v>
+        <v>16</v>
       </c>
-      <c r="B44" s="33" t="s">
-        <v>62</v>
+      <c r="B44" s="31" t="s">
+        <v>106</v>
       </c>
       <c r="C44" s="31" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="D44" s="31" t="s">
-        <v>64</v>
+        <v>109</v>
       </c>
-      <c r="E44" s="31" t="s">
-        <v>233</v>
-      </c>
+      <c r="E44" s="31"/>
       <c r="F44" s="31"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B45" s="31" t="s">
-        <v>106</v>
+      <c r="B45" s="33" t="s">
+        <v>17</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>108</v>
+        <v>48</v>
       </c>
       <c r="D45" s="31" t="s">
-        <v>109</v>
+        <v>26</v>
       </c>
       <c r="E45" s="31"/>
       <c r="F45" s="31"/>
@@ -2467,14 +2461,14 @@
       <c r="A46" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B46" s="33" t="s">
-        <v>17</v>
+      <c r="B46" s="31" t="s">
+        <v>19</v>
       </c>
       <c r="C46" s="31" t="s">
-        <v>48</v>
+        <v>157</v>
       </c>
       <c r="D46" s="31" t="s">
-        <v>26</v>
+        <v>221</v>
       </c>
       <c r="E46" s="31"/>
       <c r="F46" s="31"/>
@@ -2484,13 +2478,13 @@
         <v>16</v>
       </c>
       <c r="B47" s="31" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C47" s="31" t="s">
-        <v>159</v>
+        <v>52</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="E47" s="31"/>
       <c r="F47" s="31"/>
@@ -2500,99 +2494,95 @@
         <v>16</v>
       </c>
       <c r="B48" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C48" s="31" t="s">
-        <v>52</v>
+        <v>141</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E48" s="31"/>
       <c r="F48" s="31"/>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A49" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B49" s="31" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
-      <c r="C49" s="31" t="s">
-        <v>143</v>
+      <c r="C49" s="3" t="s">
+        <v>154</v>
       </c>
-      <c r="D49" s="31" t="s">
+      <c r="D49" s="3" t="s">
         <v>225</v>
       </c>
       <c r="E49" s="31"/>
       <c r="F49" s="31"/>
     </row>
-    <row r="50" spans="1:6" ht="56" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A50" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B50" s="31" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>227</v>
       </c>
       <c r="E50" s="31"/>
-      <c r="F50" s="34" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" ht="56" x14ac:dyDescent="0.2">
+      <c r="F50" s="31"/>
+    </row>
+    <row r="51" spans="1:6" ht="84" x14ac:dyDescent="0.2">
       <c r="A51" s="31" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="B51" s="31" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>157</v>
+        <v>228</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>229</v>
+        <v>56</v>
       </c>
-      <c r="E51" s="31"/>
-      <c r="F51" s="34" t="s">
-        <v>228</v>
+      <c r="E51" s="34" t="s">
+        <v>233</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="84" x14ac:dyDescent="0.2">
+      <c r="F51" s="31"/>
+    </row>
+    <row r="52" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A52" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B52" s="31" t="s">
-        <v>55</v>
+      <c r="B52" s="35" t="s">
+        <v>95</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>230</v>
+        <v>158</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>56</v>
+        <v>103</v>
       </c>
-      <c r="E52" s="34" t="s">
-        <v>235</v>
-      </c>
+      <c r="E52" s="31"/>
       <c r="F52" s="31"/>
     </row>
-    <row r="53" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B53" s="35" t="s">
-        <v>95</v>
+      <c r="B53" s="31" t="s">
+        <v>120</v>
       </c>
-      <c r="C53" s="3" t="s">
-        <v>160</v>
+      <c r="C53" s="31" t="s">
+        <v>144</v>
       </c>
-      <c r="D53" s="3" t="s">
-        <v>103</v>
+      <c r="D53" s="31" t="s">
+        <v>229</v>
       </c>
       <c r="E53" s="31"/>
       <c r="F53" s="31"/>
@@ -2602,15 +2592,17 @@
         <v>27</v>
       </c>
       <c r="B54" s="31" t="s">
-        <v>121</v>
+        <v>101</v>
       </c>
       <c r="C54" s="31" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D54" s="31" t="s">
-        <v>231</v>
+        <v>104</v>
       </c>
-      <c r="E54" s="31"/>
+      <c r="E54" s="31" t="s">
+        <v>230</v>
+      </c>
       <c r="F54" s="31"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -2618,51 +2610,49 @@
         <v>27</v>
       </c>
       <c r="B55" s="31" t="s">
-        <v>101</v>
+        <v>124</v>
       </c>
       <c r="C55" s="31" t="s">
-        <v>147</v>
+        <v>244</v>
       </c>
       <c r="D55" s="31" t="s">
-        <v>104</v>
+        <v>186</v>
       </c>
-      <c r="E55" s="31" t="s">
-        <v>232</v>
-      </c>
+      <c r="E55" s="31"/>
       <c r="F55" s="31"/>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B56" s="31" t="s">
-        <v>125</v>
+      <c r="B56" s="21" t="s">
+        <v>102</v>
       </c>
       <c r="C56" s="31" t="s">
-        <v>246</v>
+        <v>151</v>
       </c>
       <c r="D56" s="31" t="s">
-        <v>188</v>
+        <v>105</v>
       </c>
-      <c r="E56" s="31"/>
+      <c r="E56" s="31" t="s">
+        <v>238</v>
+      </c>
       <c r="F56" s="31"/>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B57" s="21" t="s">
-        <v>102</v>
+      <c r="B57" s="31" t="s">
+        <v>121</v>
       </c>
       <c r="C57" s="31" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
       <c r="D57" s="31" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
-      <c r="E57" s="31" t="s">
-        <v>240</v>
-      </c>
+      <c r="E57" s="31"/>
       <c r="F57" s="31"/>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.2">
@@ -2673,26 +2663,26 @@
         <v>122</v>
       </c>
       <c r="C58" s="31" t="s">
-        <v>148</v>
+        <v>234</v>
       </c>
       <c r="D58" s="31" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="E58" s="31"/>
       <c r="F58" s="31"/>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A59" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B59" s="31" t="s">
-        <v>123</v>
+      <c r="B59" s="21" t="s">
+        <v>125</v>
       </c>
       <c r="C59" s="31" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
-      <c r="D59" s="31" t="s">
-        <v>239</v>
+      <c r="D59" s="34" t="s">
+        <v>128</v>
       </c>
       <c r="E59" s="31"/>
       <c r="F59" s="31"/>
@@ -2705,7 +2695,7 @@
         <v>126</v>
       </c>
       <c r="C60" s="31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D60" s="34" t="s">
         <v>129</v>
@@ -2713,50 +2703,54 @@
       <c r="E60" s="31"/>
       <c r="F60" s="31"/>
     </row>
-    <row r="61" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A61" s="31" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
-      <c r="B61" s="21" t="s">
-        <v>127</v>
+      <c r="B61" s="31" t="s">
+        <v>28</v>
       </c>
       <c r="C61" s="31" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
-      <c r="D61" s="34" t="s">
-        <v>130</v>
+      <c r="D61" s="31" t="s">
+        <v>41</v>
       </c>
       <c r="E61" s="31"/>
-      <c r="F61" s="31"/>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F61" s="34" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="56" x14ac:dyDescent="0.2">
       <c r="A62" s="31" t="s">
         <v>29</v>
       </c>
       <c r="B62" s="31" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C62" s="31" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D62" s="31" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E62" s="31"/>
-      <c r="F62" s="31"/>
+      <c r="F62" s="34" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="31" t="s">
         <v>29</v>
       </c>
       <c r="B63" s="31" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C63" s="31" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D63" s="31" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E63" s="31"/>
       <c r="F63" s="31"/>
@@ -2766,13 +2760,13 @@
         <v>29</v>
       </c>
       <c r="B64" s="31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C64" s="31" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D64" s="31" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E64" s="31"/>
       <c r="F64" s="31"/>
@@ -2782,13 +2776,13 @@
         <v>29</v>
       </c>
       <c r="B65" s="31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C65" s="31" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D65" s="31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E65" s="31"/>
       <c r="F65" s="31"/>
@@ -2798,49 +2792,49 @@
         <v>29</v>
       </c>
       <c r="B66" s="31" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C66" s="31" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D66" s="31" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E66" s="31"/>
       <c r="F66" s="31"/>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A67" s="31" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
-      <c r="B67" s="31" t="s">
-        <v>34</v>
+      <c r="B67" s="21" t="s">
+        <v>184</v>
       </c>
       <c r="C67" s="31" t="s">
-        <v>251</v>
+        <v>185</v>
       </c>
-      <c r="D67" s="31" t="s">
-        <v>46</v>
+      <c r="D67" s="34" t="s">
+        <v>187</v>
       </c>
-      <c r="E67" s="31"/>
+      <c r="E67" s="31" t="s">
+        <v>239</v>
+      </c>
       <c r="F67" s="31"/>
     </row>
-    <row r="68" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="31" t="s">
         <v>38</v>
       </c>
-      <c r="B68" s="21" t="s">
-        <v>186</v>
+      <c r="B68" s="31" t="s">
+        <v>35</v>
       </c>
       <c r="C68" s="31" t="s">
-        <v>187</v>
+        <v>250</v>
       </c>
-      <c r="D68" s="34" t="s">
-        <v>189</v>
+      <c r="D68" s="31" t="s">
+        <v>49</v>
       </c>
-      <c r="E68" s="31" t="s">
-        <v>241</v>
-      </c>
+      <c r="E68" s="31"/>
       <c r="F68" s="31"/>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.2">
@@ -2848,13 +2842,13 @@
         <v>38</v>
       </c>
       <c r="B69" s="31" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C69" s="31" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D69" s="31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E69" s="31"/>
       <c r="F69" s="31"/>
@@ -2864,13 +2858,13 @@
         <v>38</v>
       </c>
       <c r="B70" s="31" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C70" s="31" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D70" s="31" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E70" s="31"/>
       <c r="F70" s="31"/>
@@ -2880,13 +2874,13 @@
         <v>38</v>
       </c>
       <c r="B71" s="31" t="s">
-        <v>37</v>
+        <v>188</v>
       </c>
       <c r="C71" s="31" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D71" s="31" t="s">
-        <v>51</v>
+        <v>189</v>
       </c>
       <c r="E71" s="31"/>
       <c r="F71" s="31"/>
@@ -2899,7 +2893,7 @@
         <v>190</v>
       </c>
       <c r="C72" s="31" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="D72" s="31" t="s">
         <v>191</v>
@@ -2912,32 +2906,52 @@
         <v>38</v>
       </c>
       <c r="B73" s="31" t="s">
-        <v>192</v>
+        <v>130</v>
       </c>
       <c r="C73" s="31" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D73" s="31" t="s">
-        <v>193</v>
+        <v>131</v>
       </c>
       <c r="E73" s="31"/>
       <c r="F73" s="31"/>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A74" s="31" t="s">
-        <v>38</v>
-      </c>
-      <c r="B74" s="31" t="s">
-        <v>131</v>
-      </c>
-      <c r="C74" s="31" t="s">
-        <v>256</v>
-      </c>
-      <c r="D74" s="31" t="s">
-        <v>132</v>
-      </c>
-      <c r="E74" s="31"/>
       <c r="F74" s="31"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F75" s="31"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F76" s="31"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F77" s="31"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F78" s="31"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F79" s="31"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="F80" s="31"/>
+    </row>
+    <row r="81" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F81" s="31"/>
+    </row>
+    <row r="82" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F82" s="31"/>
+    </row>
+    <row r="83" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F83" s="31"/>
+    </row>
+    <row r="84" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F84" s="31"/>
+    </row>
+    <row r="85" spans="6:6" x14ac:dyDescent="0.2">
+      <c r="F85" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2960,12 +2974,12 @@
   <sheetData>
     <row r="1" spans="1:4" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
@@ -2981,18 +2995,18 @@
       <c r="B3" s="46"/>
       <c r="C3" s="46"/>
       <c r="D3" s="11" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -3026,12 +3040,12 @@
   <sheetData>
     <row r="1" spans="1:15" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="10" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -3052,7 +3066,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="15" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B4" s="16" t="s">
         <v>66</v>
@@ -3070,16 +3084,16 @@
         <v>70</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>71</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>72</v>
@@ -3091,7 +3105,7 @@
         <v>74</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>75</v>
@@ -44038,12 +44052,12 @@
   <sheetData>
     <row r="1" spans="1:53" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="46" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B1" s="47"/>
       <c r="C1" s="47"/>
       <c r="D1" s="5" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
@@ -44064,7 +44078,7 @@
     </row>
     <row r="4" spans="1:53" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="X4" t="s">
         <v>16</v>
@@ -44087,10 +44101,10 @@
         <v>65</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>53</v>
@@ -44099,13 +44113,13 @@
         <v>96</v>
       </c>
       <c r="G5" s="37" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="I5" s="39" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J5" s="37" t="s">
         <v>15</v>
@@ -44114,7 +44128,7 @@
         <v>107</v>
       </c>
       <c r="L5" s="37" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="M5" s="37" t="s">
         <v>8</v>
@@ -44123,10 +44137,10 @@
         <v>13</v>
       </c>
       <c r="O5" s="37" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="P5" s="37" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="Q5" s="37" t="s">
         <v>99</v>
@@ -44135,13 +44149,13 @@
         <v>100</v>
       </c>
       <c r="S5" s="37" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="T5" s="40" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="U5" s="40" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="V5" s="39" t="s">
         <v>9</v>
@@ -44165,10 +44179,10 @@
         <v>21</v>
       </c>
       <c r="AC5" s="42" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="AD5" s="42" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="AE5" s="42" t="s">
         <v>55</v>
@@ -44177,28 +44191,28 @@
         <v>95</v>
       </c>
       <c r="AG5" s="37" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="AH5" s="37" t="s">
         <v>101</v>
       </c>
       <c r="AI5" s="37" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="AJ5" s="37" t="s">
         <v>102</v>
       </c>
       <c r="AK5" s="40" t="s">
+        <v>121</v>
+      </c>
+      <c r="AL5" s="40" t="s">
         <v>122</v>
       </c>
-      <c r="AL5" s="40" t="s">
-        <v>123</v>
-      </c>
       <c r="AM5" s="40" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="AN5" s="40" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="AO5" s="37" t="s">
         <v>28</v>
@@ -44219,7 +44233,7 @@
         <v>34</v>
       </c>
       <c r="AU5" s="37" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AV5" s="37" t="s">
         <v>35</v>
@@ -44231,13 +44245,13 @@
         <v>37</v>
       </c>
       <c r="AY5" s="37" t="s">
+        <v>188</v>
+      </c>
+      <c r="AZ5" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="AZ5" s="37" t="s">
-        <v>192</v>
-      </c>
       <c r="BA5" s="37" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
follow insuite template 20
</commit_message>
<xml_diff>
--- a/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
+++ b/www/data-entry-template/GLATAR_data_entry_template_v20.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benhlina/Library/CloudStorage/Dropbox/GitHub/GLATAR-App/www/data-entry-template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D94E3D2A-47E0-E844-8BF2-DA05771D155A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{589E0174-896C-4C40-A4AE-F760894775D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="19460" xr2:uid="{DE6F8925-643B-304C-8933-23D4A9123DA3}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -2427,34 +2427,36 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="31" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
       <c r="B44" s="31" t="s">
-        <v>106</v>
+        <v>120</v>
       </c>
       <c r="C44" s="31" t="s">
-        <v>108</v>
+        <v>144</v>
       </c>
       <c r="D44" s="31" t="s">
-        <v>109</v>
+        <v>229</v>
       </c>
       <c r="E44" s="31"/>
       <c r="F44" s="31"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="31" t="s">
-        <v>16</v>
+        <v>123</v>
       </c>
-      <c r="B45" s="33" t="s">
-        <v>17</v>
+      <c r="B45" s="31" t="s">
+        <v>101</v>
       </c>
       <c r="C45" s="31" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
       <c r="D45" s="31" t="s">
-        <v>26</v>
+        <v>104</v>
       </c>
-      <c r="E45" s="31"/>
+      <c r="E45" s="31" t="s">
+        <v>230</v>
+      </c>
       <c r="F45" s="31"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
@@ -2462,13 +2464,13 @@
         <v>16</v>
       </c>
       <c r="B46" s="31" t="s">
-        <v>19</v>
+        <v>106</v>
       </c>
       <c r="C46" s="31" t="s">
-        <v>157</v>
+        <v>108</v>
       </c>
       <c r="D46" s="31" t="s">
-        <v>221</v>
+        <v>109</v>
       </c>
       <c r="E46" s="31"/>
       <c r="F46" s="31"/>
@@ -2477,14 +2479,14 @@
       <c r="A47" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B47" s="31" t="s">
-        <v>20</v>
+      <c r="B47" s="33" t="s">
+        <v>17</v>
       </c>
       <c r="C47" s="31" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D47" s="31" t="s">
-        <v>222</v>
+        <v>26</v>
       </c>
       <c r="E47" s="31"/>
       <c r="F47" s="31"/>
@@ -2494,115 +2496,113 @@
         <v>16</v>
       </c>
       <c r="B48" s="31" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C48" s="31" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="D48" s="31" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E48" s="31"/>
       <c r="F48" s="31"/>
     </row>
-    <row r="49" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B49" s="31" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
-      <c r="C49" s="3" t="s">
-        <v>154</v>
+      <c r="C49" s="31" t="s">
+        <v>52</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>225</v>
+      <c r="D49" s="31" t="s">
+        <v>222</v>
       </c>
       <c r="E49" s="31"/>
       <c r="F49" s="31"/>
     </row>
-    <row r="50" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="31" t="s">
         <v>16</v>
       </c>
       <c r="B50" s="31" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
-      <c r="C50" s="3" t="s">
-        <v>155</v>
+      <c r="C50" s="31" t="s">
+        <v>141</v>
       </c>
-      <c r="D50" s="3" t="s">
-        <v>227</v>
+      <c r="D50" s="31" t="s">
+        <v>223</v>
       </c>
       <c r="E50" s="31"/>
       <c r="F50" s="31"/>
     </row>
-    <row r="51" spans="1:6" ht="84" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A51" s="31" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="B51" s="31" t="s">
-        <v>55</v>
+        <v>22</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>228</v>
+        <v>154</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>56</v>
+        <v>225</v>
       </c>
-      <c r="E51" s="34" t="s">
-        <v>233</v>
-      </c>
+      <c r="E51" s="31"/>
       <c r="F51" s="31"/>
     </row>
     <row r="52" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A52" s="31" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
-      <c r="B52" s="35" t="s">
-        <v>95</v>
+      <c r="B52" s="31" t="s">
+        <v>23</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>103</v>
+        <v>227</v>
       </c>
       <c r="E52" s="31"/>
       <c r="F52" s="31"/>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" ht="84" x14ac:dyDescent="0.2">
       <c r="A53" s="31" t="s">
         <v>27</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
-      <c r="C53" s="31" t="s">
-        <v>144</v>
+      <c r="C53" s="3" t="s">
+        <v>228</v>
       </c>
-      <c r="D53" s="31" t="s">
-        <v>229</v>
+      <c r="D53" s="3" t="s">
+        <v>56</v>
       </c>
-      <c r="E53" s="31"/>
+      <c r="E53" s="34" t="s">
+        <v>233</v>
+      </c>
       <c r="F53" s="31"/>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" ht="28" x14ac:dyDescent="0.2">
       <c r="A54" s="31" t="s">
         <v>27</v>
       </c>
-      <c r="B54" s="31" t="s">
-        <v>101</v>
+      <c r="B54" s="35" t="s">
+        <v>95</v>
       </c>
-      <c r="C54" s="31" t="s">
-        <v>145</v>
+      <c r="C54" s="3" t="s">
+        <v>158</v>
       </c>
-      <c r="D54" s="31" t="s">
-        <v>104</v>
+      <c r="D54" s="3" t="s">
+        <v>103</v>
       </c>
-      <c r="E54" s="31" t="s">
-        <v>230</v>
-      </c>
+      <c r="E54" s="31"/>
       <c r="F54" s="31"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.2">
@@ -44035,14 +44035,14 @@
     <col min="20" max="20" width="9" style="8" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="15.5" style="8" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.5" customWidth="1"/>
-    <col min="28" max="28" width="10.83203125" customWidth="1"/>
-    <col min="29" max="29" width="22.6640625" customWidth="1"/>
-    <col min="30" max="30" width="31.1640625" customWidth="1"/>
-    <col min="31" max="31" width="17.5" customWidth="1"/>
-    <col min="32" max="32" width="27" customWidth="1"/>
-    <col min="33" max="33" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.5" customWidth="1"/>
+    <col min="30" max="30" width="10.83203125" customWidth="1"/>
+    <col min="31" max="31" width="22.6640625" customWidth="1"/>
+    <col min="32" max="32" width="31.1640625" customWidth="1"/>
+    <col min="33" max="33" width="17.5" customWidth="1"/>
+    <col min="34" max="34" width="27" customWidth="1"/>
     <col min="35" max="35" width="18.1640625" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="42" max="45" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -44080,10 +44080,10 @@
       <c r="A4" t="s">
         <v>123</v>
       </c>
-      <c r="X4" t="s">
+      <c r="Z4" t="s">
         <v>16</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AG4" t="s">
         <v>27</v>
       </c>
       <c r="AO4" t="s">
@@ -44163,38 +44163,38 @@
       <c r="W5" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="X5" s="40" t="s">
+      <c r="X5" s="37" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y5" s="37" t="s">
+        <v>101</v>
+      </c>
+      <c r="Z5" s="40" t="s">
         <v>106</v>
       </c>
-      <c r="Y5" s="39" t="s">
+      <c r="AA5" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="Z5" s="37" t="s">
+      <c r="AB5" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="AA5" s="37" t="s">
+      <c r="AC5" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="AB5" s="37" t="s">
+      <c r="AD5" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="AC5" s="42" t="s">
+      <c r="AE5" s="42" t="s">
         <v>170</v>
       </c>
-      <c r="AD5" s="42" t="s">
+      <c r="AF5" s="42" t="s">
         <v>171</v>
       </c>
-      <c r="AE5" s="42" t="s">
+      <c r="AG5" s="42" t="s">
         <v>55</v>
       </c>
-      <c r="AF5" s="42" t="s">
+      <c r="AH5" s="42" t="s">
         <v>95</v>
-      </c>
-      <c r="AG5" s="37" t="s">
-        <v>120</v>
-      </c>
-      <c r="AH5" s="37" t="s">
-        <v>101</v>
       </c>
       <c r="AI5" s="37" t="s">
         <v>124</v>
@@ -44273,13 +44273,13 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="W6:W999" xr:uid="{618BEA16-FB85-144A-9DB4-305EFF123E53}">
       <formula1>"wet, dried"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH6:AH999" xr:uid="{66E4A2BE-9678-EC4D-BD77-D6B9C6555CFA}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y6:Y999" xr:uid="{66E4A2BE-9678-EC4D-BD77-D6B9C6555CFA}">
       <formula1>"wet, dry"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AI1001:AI9999 AJ6:AJ1000" xr:uid="{E08CD4DA-AE11-DB40-922E-0C3ECAF74329}">
       <formula1>"Joules/g"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE6:AE1000" xr:uid="{9917EF8E-9D15-EA4E-B86B-60B39CF888A1}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AG6:AG1000" xr:uid="{9917EF8E-9D15-EA4E-B86B-60B39CF888A1}">
       <formula1>"Parr oxygen bomb, Parr semi-micro oxygen bomb, Phillipson microbomb, Gentry-Weigert bomb, Unknown bomb, Proximate composition, Organic analysis, Wet digestion, Unknown"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V6:V10000" xr:uid="{783A5061-181E-6647-B48C-F16794E29794}">
@@ -44291,7 +44291,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T6:T10000" xr:uid="{FE3B4961-9F35-5942-85C0-C97B5B164DB5}">
       <formula1>"Idividual, Composite, Mean, SD, Equation"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M7:M10000 M6" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M6:M10000" xr:uid="{D77F31B9-1615-2E41-A61E-3373EC534A30}">
       <formula1>"fry, larva, nymph, pupa, juvenile, adult "</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L6:L10000" xr:uid="{8E9C54B4-F117-8C42-9731-37E4B818ABAE}">

</xml_diff>